<commit_message>
FIF-093 Saxo fixtures carry all three sheets
The anonymizer now reads and writes Transacties, _Transacties and
Bookings, each with its own header row and row count, and the five
committed Saxo fixtures are regenerated with all three sheets present.
Join keys survive anonymization and are asserted to, and a booking's
components still sum to it after perturbation.

Requirements: TST-031, TST-012, TST-013, TST-028, TST-029

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/saxo-nl/Transactions_10000000_2021-11-29_2021-12-31.xlsx
+++ b/fixtures/saxo-nl/Transactions_10000000_2021-11-29_2021-12-31.xlsx
@@ -8,13 +8,15 @@
   </bookViews>
   <sheets>
     <sheet name="Transacties" sheetId="1" r:id="rId1"/>
+    <sheet name="_Transacties" sheetId="2" r:id="rId2"/>
+    <sheet name="Bookings" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="182">
   <si>
     <t>Klant-id</t>
   </si>
@@ -151,315 +153,424 @@
     <t>40100/9000001EUR</t>
   </si>
   <si>
+    <t>40000000065</t>
+  </si>
+  <si>
+    <t>Geldoverboeking</t>
+  </si>
+  <si>
+    <t>Service fee</t>
+  </si>
+  <si>
+    <t>Cash</t>
+  </si>
+  <si>
+    <t>5000003</t>
+  </si>
+  <si>
+    <t>2500000000</t>
+  </si>
+  <si>
+    <t>40000000026</t>
+  </si>
+  <si>
+    <t>Storting</t>
+  </si>
+  <si>
+    <t>Unknown</t>
+  </si>
+  <si>
+    <t>40100/9000001USD</t>
+  </si>
+  <si>
+    <t>2500000034</t>
+  </si>
+  <si>
+    <t>40000000013</t>
+  </si>
+  <si>
+    <t>USD</t>
+  </si>
+  <si>
+    <t>2500000017</t>
+  </si>
+  <si>
+    <t>40000000000</t>
+  </si>
+  <si>
+    <t>7000000007</t>
+  </si>
+  <si>
+    <t>2500000051</t>
+  </si>
+  <si>
+    <t>Transactie</t>
+  </si>
+  <si>
+    <t>Deponering 3000 @ 138.00 EUR</t>
+  </si>
+  <si>
+    <t>Fixture Instrument 04</t>
+  </si>
+  <si>
+    <t>FXT06</t>
+  </si>
+  <si>
+    <t>XF0000000103</t>
+  </si>
+  <si>
+    <t>Bond</t>
+  </si>
+  <si>
+    <t>Euronext Amsterdam Bonds</t>
+  </si>
+  <si>
+    <t>7000000014</t>
+  </si>
+  <si>
+    <t>2500000068</t>
+  </si>
+  <si>
+    <t>Deponering 30 @ 37.47 EUR</t>
+  </si>
+  <si>
+    <t>Fixture Instrument 11</t>
+  </si>
+  <si>
+    <t>FXT08:xams</t>
+  </si>
+  <si>
+    <t>XF0000000095</t>
+  </si>
+  <si>
+    <t>Euronext Amsterdam</t>
+  </si>
+  <si>
+    <t>7000000021</t>
+  </si>
+  <si>
+    <t>2500000085</t>
+  </si>
+  <si>
+    <t>Deponering 4 @ 87.86 EUR</t>
+  </si>
+  <si>
+    <t>Fixture Instrument 10</t>
+  </si>
+  <si>
+    <t>FXT07</t>
+  </si>
+  <si>
+    <t>XF0000000129</t>
+  </si>
+  <si>
+    <t>MutualFund</t>
+  </si>
+  <si>
+    <t>Euronext Amsterdam Funds</t>
+  </si>
+  <si>
+    <t>7000000028</t>
+  </si>
+  <si>
+    <t>2500000102</t>
+  </si>
+  <si>
+    <t>Deponering 2000 @ 81.00 EUR</t>
+  </si>
+  <si>
+    <t>Fixture Instrument 00</t>
+  </si>
+  <si>
+    <t>FXT15</t>
+  </si>
+  <si>
+    <t>XF0000000178</t>
+  </si>
+  <si>
+    <t>Generic Bonds exchange</t>
+  </si>
+  <si>
+    <t>7000000063</t>
+  </si>
+  <si>
+    <t>2500000187</t>
+  </si>
+  <si>
+    <t>Deponering 3 @ 11.80 EUR</t>
+  </si>
+  <si>
+    <t>Fixture Instrument 03</t>
+  </si>
+  <si>
+    <t>FXT03:xams</t>
+  </si>
+  <si>
+    <t>XF0000000087</t>
+  </si>
+  <si>
+    <t>7000000070</t>
+  </si>
+  <si>
+    <t>2500000204</t>
+  </si>
+  <si>
+    <t>Deponering 15 @ 151.57 USD</t>
+  </si>
+  <si>
+    <t>Fixture Instrument 12</t>
+  </si>
+  <si>
+    <t>FXT13:xnas</t>
+  </si>
+  <si>
+    <t>XF0000000160</t>
+  </si>
+  <si>
+    <t>NASDAQ</t>
+  </si>
+  <si>
+    <t>7000000042</t>
+  </si>
+  <si>
+    <t>2500000136</t>
+  </si>
+  <si>
+    <t>Deponering 3 @ 31.75 EUR</t>
+  </si>
+  <si>
+    <t>Fixture Instrument 02</t>
+  </si>
+  <si>
+    <t>FXT01:xams</t>
+  </si>
+  <si>
+    <t>XF0000000111</t>
+  </si>
+  <si>
+    <t>7000000077</t>
+  </si>
+  <si>
+    <t>2500000221</t>
+  </si>
+  <si>
+    <t>Deponering 100 @ 18.53 EUR</t>
+  </si>
+  <si>
+    <t>Fixture Instrument 15</t>
+  </si>
+  <si>
+    <t>FXT11:xetr</t>
+  </si>
+  <si>
+    <t>XF0000000061</t>
+  </si>
+  <si>
+    <t>Etf</t>
+  </si>
+  <si>
+    <t>Deutsche Börse (Indices &amp; ETFs)</t>
+  </si>
+  <si>
+    <t>7000000049</t>
+  </si>
+  <si>
+    <t>2500000153</t>
+  </si>
+  <si>
+    <t>Deponering 60 @ 30.33 EUR</t>
+  </si>
+  <si>
+    <t>Fixture Instrument 16</t>
+  </si>
+  <si>
+    <t>FXT00:xams</t>
+  </si>
+  <si>
+    <t>XF0000000046</t>
+  </si>
+  <si>
+    <t>7000000056</t>
+  </si>
+  <si>
+    <t>2500000170</t>
+  </si>
+  <si>
+    <t>Deponering 345 @ 6.59 EUR</t>
+  </si>
+  <si>
+    <t>Fixture Instrument 18</t>
+  </si>
+  <si>
+    <t>FXT09:xetr</t>
+  </si>
+  <si>
+    <t>XF0000000053</t>
+  </si>
+  <si>
+    <t>7000000035</t>
+  </si>
+  <si>
+    <t>2500000119</t>
+  </si>
+  <si>
+    <t>Deponering 300 @ 51.64 EUR</t>
+  </si>
+  <si>
+    <t>Fixture Instrument 17</t>
+  </si>
+  <si>
+    <t>FXT02:xams</t>
+  </si>
+  <si>
+    <t>XF0000000038</t>
+  </si>
+  <si>
+    <t>7000000000</t>
+  </si>
+  <si>
+    <t>2500000238</t>
+  </si>
+  <si>
+    <t>Deponering 3 @ 179.07 USD</t>
+  </si>
+  <si>
+    <t>*Delisted 20231002 (Fixture Instrument 07)</t>
+  </si>
+  <si>
+    <t>FXT04:xbru</t>
+  </si>
+  <si>
+    <t>XF0000000145</t>
+  </si>
+  <si>
+    <t>Euronext Brussels</t>
+  </si>
+  <si>
+    <t>7000000084</t>
+  </si>
+  <si>
+    <t>2500000255</t>
+  </si>
+  <si>
+    <t>Deponering 300 @ 14.25 CAD</t>
+  </si>
+  <si>
+    <t>Order-ID</t>
+  </si>
+  <si>
+    <t>Aangepaste transactiedatum</t>
+  </si>
+  <si>
+    <t>Uitvoeringsdatum transactie</t>
+  </si>
+  <si>
+    <t>Trade Event Type</t>
+  </si>
+  <si>
+    <t>Trade Type</t>
+  </si>
+  <si>
+    <t>Openen/sluiten</t>
+  </si>
+  <si>
+    <t>Traded Quantity</t>
+  </si>
+  <si>
+    <t>Prijs</t>
+  </si>
+  <si>
+    <t>Verhandelde waarde</t>
+  </si>
+  <si>
+    <t>Spreadkosten</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>Deponering</t>
+  </si>
+  <si>
+    <t>NotAvailable</t>
+  </si>
+  <si>
+    <t>Te openen</t>
+  </si>
+  <si>
+    <t>Amount Type</t>
+  </si>
+  <si>
+    <t>Amount Type Id</t>
+  </si>
+  <si>
+    <t>Boekingsdatum</t>
+  </si>
+  <si>
+    <t>Ex-datum</t>
+  </si>
+  <si>
+    <t>Boekdatum</t>
+  </si>
+  <si>
+    <t>In aanmerking komend aantal</t>
+  </si>
+  <si>
+    <t>Dividend per aandeel</t>
+  </si>
+  <si>
+    <t>Tax Percentage</t>
+  </si>
+  <si>
+    <t>40000000091</t>
+  </si>
+  <si>
+    <t>Corporate actions - Voorheffing</t>
+  </si>
+  <si>
+    <t>55</t>
+  </si>
+  <si>
+    <t>14-dec-2021</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>40000000078</t>
+  </si>
+  <si>
+    <t>Corporate Actions - Cashdividenden</t>
+  </si>
+  <si>
+    <t>56</t>
+  </si>
+  <si>
+    <t>0.09 CAD</t>
+  </si>
+  <si>
+    <t>477</t>
+  </si>
+  <si>
+    <t>40000000052</t>
+  </si>
+  <si>
+    <t>12-nov-2021</t>
+  </si>
+  <si>
     <t>40000000039</t>
   </si>
   <si>
-    <t>Geldoverboeking</t>
-  </si>
-  <si>
-    <t>Service fee</t>
-  </si>
-  <si>
-    <t>Cash</t>
-  </si>
-  <si>
-    <t>5000003</t>
-  </si>
-  <si>
-    <t>2500000000</t>
-  </si>
-  <si>
-    <t>40000000026</t>
-  </si>
-  <si>
-    <t>Storting</t>
-  </si>
-  <si>
-    <t>Unknown</t>
-  </si>
-  <si>
-    <t>40100/9000001USD</t>
-  </si>
-  <si>
-    <t>2500000034</t>
-  </si>
-  <si>
-    <t>40000000013</t>
-  </si>
-  <si>
-    <t>USD</t>
-  </si>
-  <si>
-    <t>2500000017</t>
-  </si>
-  <si>
-    <t>40000000000</t>
-  </si>
-  <si>
-    <t>7000000007</t>
-  </si>
-  <si>
-    <t>2500000051</t>
-  </si>
-  <si>
-    <t>Transactie</t>
-  </si>
-  <si>
-    <t>Deponering 3000 @ 138.00 EUR</t>
-  </si>
-  <si>
-    <t>Fixture Instrument 04</t>
-  </si>
-  <si>
-    <t>FXT06</t>
-  </si>
-  <si>
-    <t>XF0000000103</t>
-  </si>
-  <si>
-    <t>Bond</t>
-  </si>
-  <si>
-    <t>Euronext Amsterdam Bonds</t>
-  </si>
-  <si>
-    <t>7000000014</t>
-  </si>
-  <si>
-    <t>2500000068</t>
-  </si>
-  <si>
-    <t>Deponering 30 @ 37.47 EUR</t>
-  </si>
-  <si>
-    <t>Fixture Instrument 11</t>
-  </si>
-  <si>
-    <t>FXT08:xams</t>
-  </si>
-  <si>
-    <t>XF0000000095</t>
-  </si>
-  <si>
-    <t>Euronext Amsterdam</t>
-  </si>
-  <si>
-    <t>7000000021</t>
-  </si>
-  <si>
-    <t>2500000085</t>
-  </si>
-  <si>
-    <t>Deponering 4 @ 87.86 EUR</t>
-  </si>
-  <si>
-    <t>Fixture Instrument 10</t>
-  </si>
-  <si>
-    <t>FXT07</t>
-  </si>
-  <si>
-    <t>XF0000000129</t>
-  </si>
-  <si>
-    <t>MutualFund</t>
-  </si>
-  <si>
-    <t>Euronext Amsterdam Funds</t>
-  </si>
-  <si>
-    <t>7000000028</t>
-  </si>
-  <si>
-    <t>2500000102</t>
-  </si>
-  <si>
-    <t>Deponering 2000 @ 81.00 EUR</t>
-  </si>
-  <si>
-    <t>Fixture Instrument 00</t>
-  </si>
-  <si>
-    <t>FXT15</t>
-  </si>
-  <si>
-    <t>XF0000000178</t>
-  </si>
-  <si>
-    <t>Generic Bonds exchange</t>
-  </si>
-  <si>
-    <t>7000000063</t>
-  </si>
-  <si>
-    <t>2500000187</t>
-  </si>
-  <si>
-    <t>Deponering 3 @ 11.80 EUR</t>
-  </si>
-  <si>
-    <t>Fixture Instrument 03</t>
-  </si>
-  <si>
-    <t>FXT03:xams</t>
-  </si>
-  <si>
-    <t>XF0000000087</t>
-  </si>
-  <si>
-    <t>7000000070</t>
-  </si>
-  <si>
-    <t>2500000204</t>
-  </si>
-  <si>
-    <t>Deponering 15 @ 151.57 USD</t>
-  </si>
-  <si>
-    <t>Fixture Instrument 12</t>
-  </si>
-  <si>
-    <t>FXT13:xnas</t>
-  </si>
-  <si>
-    <t>XF0000000160</t>
-  </si>
-  <si>
-    <t>NASDAQ</t>
-  </si>
-  <si>
-    <t>7000000042</t>
-  </si>
-  <si>
-    <t>2500000136</t>
-  </si>
-  <si>
-    <t>Deponering 3 @ 31.75 EUR</t>
-  </si>
-  <si>
-    <t>Fixture Instrument 02</t>
-  </si>
-  <si>
-    <t>FXT01:xams</t>
-  </si>
-  <si>
-    <t>XF0000000111</t>
-  </si>
-  <si>
-    <t>7000000077</t>
-  </si>
-  <si>
-    <t>2500000221</t>
-  </si>
-  <si>
-    <t>Deponering 100 @ 18.53 EUR</t>
-  </si>
-  <si>
-    <t>Fixture Instrument 15</t>
-  </si>
-  <si>
-    <t>FXT11:xetr</t>
-  </si>
-  <si>
-    <t>XF0000000061</t>
-  </si>
-  <si>
-    <t>Etf</t>
-  </si>
-  <si>
-    <t>Deutsche Börse (Indices &amp; ETFs)</t>
-  </si>
-  <si>
-    <t>7000000049</t>
-  </si>
-  <si>
-    <t>2500000153</t>
-  </si>
-  <si>
-    <t>Deponering 60 @ 30.33 EUR</t>
-  </si>
-  <si>
-    <t>Fixture Instrument 16</t>
-  </si>
-  <si>
-    <t>FXT00:xams</t>
-  </si>
-  <si>
-    <t>XF0000000046</t>
-  </si>
-  <si>
-    <t>7000000056</t>
-  </si>
-  <si>
-    <t>2500000170</t>
-  </si>
-  <si>
-    <t>Deponering 345 @ 6.59 EUR</t>
-  </si>
-  <si>
-    <t>Fixture Instrument 18</t>
-  </si>
-  <si>
-    <t>FXT09:xetr</t>
-  </si>
-  <si>
-    <t>XF0000000053</t>
-  </si>
-  <si>
-    <t>7000000035</t>
-  </si>
-  <si>
-    <t>2500000119</t>
-  </si>
-  <si>
-    <t>Deponering 300 @ 51.64 EUR</t>
-  </si>
-  <si>
-    <t>Fixture Instrument 17</t>
-  </si>
-  <si>
-    <t>FXT02:xams</t>
-  </si>
-  <si>
-    <t>XF0000000038</t>
-  </si>
-  <si>
-    <t>7000000000</t>
-  </si>
-  <si>
-    <t>2500000238</t>
-  </si>
-  <si>
-    <t>Deponering 3 @ 179.07 USD</t>
-  </si>
-  <si>
-    <t>*Delisted 20231002 (Fixture Instrument 07)</t>
-  </si>
-  <si>
-    <t>FXT04:xbru</t>
-  </si>
-  <si>
-    <t>XF0000000145</t>
-  </si>
-  <si>
-    <t>Euronext Brussels</t>
-  </si>
-  <si>
-    <t>7000000084</t>
-  </si>
-  <si>
-    <t>2500000255</t>
-  </si>
-  <si>
-    <t>Deponering 300 @ 14.25 CAD</t>
+    <t>76</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd-mmm-yyyy"/>
+    <numFmt numFmtId="165" formatCode="dd-mmm-yyyy hh:mm:ss"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -490,9 +601,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2132,4 +2244,1357 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:X14"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:24">
+      <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" t="s">
+        <v>146</v>
+      </c>
+      <c r="H1" t="s">
+        <v>147</v>
+      </c>
+      <c r="I1" t="s">
+        <v>148</v>
+      </c>
+      <c r="J1" t="s">
+        <v>149</v>
+      </c>
+      <c r="K1" t="s">
+        <v>150</v>
+      </c>
+      <c r="L1" t="s">
+        <v>151</v>
+      </c>
+      <c r="M1" t="s">
+        <v>152</v>
+      </c>
+      <c r="N1" t="s">
+        <v>153</v>
+      </c>
+      <c r="O1" t="s">
+        <v>154</v>
+      </c>
+      <c r="P1" t="s">
+        <v>155</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>29</v>
+      </c>
+      <c r="R1" t="s">
+        <v>30</v>
+      </c>
+      <c r="S1" t="s">
+        <v>23</v>
+      </c>
+      <c r="T1" t="s">
+        <v>24</v>
+      </c>
+      <c r="U1" t="s">
+        <v>25</v>
+      </c>
+      <c r="V1" t="s">
+        <v>26</v>
+      </c>
+      <c r="W1" t="s">
+        <v>27</v>
+      </c>
+      <c r="X1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24">
+      <c r="A2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F2" t="s">
+        <v>63</v>
+      </c>
+      <c r="G2" t="s">
+        <v>156</v>
+      </c>
+      <c r="H2" s="1">
+        <v>44529</v>
+      </c>
+      <c r="I2" s="2">
+        <v>44529.8111689815</v>
+      </c>
+      <c r="J2" t="s">
+        <v>157</v>
+      </c>
+      <c r="K2" t="s">
+        <v>158</v>
+      </c>
+      <c r="L2" t="s">
+        <v>159</v>
+      </c>
+      <c r="M2">
+        <v>3000</v>
+      </c>
+      <c r="N2">
+        <v>138</v>
+      </c>
+      <c r="O2">
+        <v>-4140</v>
+      </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>43</v>
+      </c>
+      <c r="S2" t="s">
+        <v>64</v>
+      </c>
+      <c r="T2" t="s">
+        <v>65</v>
+      </c>
+      <c r="U2" t="s">
+        <v>66</v>
+      </c>
+      <c r="V2" t="s">
+        <v>36</v>
+      </c>
+      <c r="W2" t="s">
+        <v>67</v>
+      </c>
+      <c r="X2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24">
+      <c r="A3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" t="s">
+        <v>69</v>
+      </c>
+      <c r="F3" t="s">
+        <v>71</v>
+      </c>
+      <c r="G3" t="s">
+        <v>156</v>
+      </c>
+      <c r="H3" s="1">
+        <v>44529</v>
+      </c>
+      <c r="I3" s="2">
+        <v>44529.8111689815</v>
+      </c>
+      <c r="J3" t="s">
+        <v>157</v>
+      </c>
+      <c r="K3" t="s">
+        <v>158</v>
+      </c>
+      <c r="L3" t="s">
+        <v>159</v>
+      </c>
+      <c r="M3">
+        <v>30</v>
+      </c>
+      <c r="N3">
+        <v>37.47</v>
+      </c>
+      <c r="O3">
+        <v>-1124.15</v>
+      </c>
+      <c r="P3">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>43</v>
+      </c>
+      <c r="S3" t="s">
+        <v>72</v>
+      </c>
+      <c r="T3" t="s">
+        <v>73</v>
+      </c>
+      <c r="U3" t="s">
+        <v>74</v>
+      </c>
+      <c r="V3" t="s">
+        <v>36</v>
+      </c>
+      <c r="W3" t="s">
+        <v>41</v>
+      </c>
+      <c r="X3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24">
+      <c r="A4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F4" t="s">
+        <v>78</v>
+      </c>
+      <c r="G4" t="s">
+        <v>156</v>
+      </c>
+      <c r="H4" s="1">
+        <v>44529</v>
+      </c>
+      <c r="I4" s="2">
+        <v>44529.8111689815</v>
+      </c>
+      <c r="J4" t="s">
+        <v>157</v>
+      </c>
+      <c r="K4" t="s">
+        <v>158</v>
+      </c>
+      <c r="L4" t="s">
+        <v>159</v>
+      </c>
+      <c r="M4">
+        <v>4</v>
+      </c>
+      <c r="N4">
+        <v>87.86</v>
+      </c>
+      <c r="O4">
+        <v>-351.44</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>43</v>
+      </c>
+      <c r="S4" t="s">
+        <v>79</v>
+      </c>
+      <c r="T4" t="s">
+        <v>80</v>
+      </c>
+      <c r="U4" t="s">
+        <v>81</v>
+      </c>
+      <c r="V4" t="s">
+        <v>36</v>
+      </c>
+      <c r="W4" t="s">
+        <v>82</v>
+      </c>
+      <c r="X4" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24">
+      <c r="A5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" t="s">
+        <v>84</v>
+      </c>
+      <c r="F5" t="s">
+        <v>86</v>
+      </c>
+      <c r="G5" t="s">
+        <v>156</v>
+      </c>
+      <c r="H5" s="1">
+        <v>44529</v>
+      </c>
+      <c r="I5" s="2">
+        <v>44529.8111689815</v>
+      </c>
+      <c r="J5" t="s">
+        <v>157</v>
+      </c>
+      <c r="K5" t="s">
+        <v>158</v>
+      </c>
+      <c r="L5" t="s">
+        <v>159</v>
+      </c>
+      <c r="M5">
+        <v>2000</v>
+      </c>
+      <c r="N5">
+        <v>89.2</v>
+      </c>
+      <c r="O5">
+        <v>-1784</v>
+      </c>
+      <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>43</v>
+      </c>
+      <c r="S5" t="s">
+        <v>87</v>
+      </c>
+      <c r="T5" t="s">
+        <v>88</v>
+      </c>
+      <c r="U5" t="s">
+        <v>89</v>
+      </c>
+      <c r="V5" t="s">
+        <v>36</v>
+      </c>
+      <c r="W5" t="s">
+        <v>67</v>
+      </c>
+      <c r="X5" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24">
+      <c r="A6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" t="s">
+        <v>91</v>
+      </c>
+      <c r="F6" t="s">
+        <v>93</v>
+      </c>
+      <c r="G6" t="s">
+        <v>156</v>
+      </c>
+      <c r="H6" s="1">
+        <v>44529</v>
+      </c>
+      <c r="I6" s="2">
+        <v>44529.8111689815</v>
+      </c>
+      <c r="J6" t="s">
+        <v>157</v>
+      </c>
+      <c r="K6" t="s">
+        <v>158</v>
+      </c>
+      <c r="L6" t="s">
+        <v>159</v>
+      </c>
+      <c r="M6">
+        <v>3</v>
+      </c>
+      <c r="N6">
+        <v>11.8</v>
+      </c>
+      <c r="O6">
+        <v>-35.4</v>
+      </c>
+      <c r="P6">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>43</v>
+      </c>
+      <c r="S6" t="s">
+        <v>94</v>
+      </c>
+      <c r="T6" t="s">
+        <v>95</v>
+      </c>
+      <c r="U6" t="s">
+        <v>96</v>
+      </c>
+      <c r="V6" t="s">
+        <v>36</v>
+      </c>
+      <c r="W6" t="s">
+        <v>41</v>
+      </c>
+      <c r="X6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24">
+      <c r="A7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" t="s">
+        <v>97</v>
+      </c>
+      <c r="F7" t="s">
+        <v>99</v>
+      </c>
+      <c r="G7" t="s">
+        <v>156</v>
+      </c>
+      <c r="H7" s="1">
+        <v>44529</v>
+      </c>
+      <c r="I7" s="2">
+        <v>44529.8111689815</v>
+      </c>
+      <c r="J7" t="s">
+        <v>157</v>
+      </c>
+      <c r="K7" t="s">
+        <v>158</v>
+      </c>
+      <c r="L7" t="s">
+        <v>159</v>
+      </c>
+      <c r="M7">
+        <v>15</v>
+      </c>
+      <c r="N7">
+        <v>151.57</v>
+      </c>
+      <c r="O7">
+        <v>-2273.56</v>
+      </c>
+      <c r="P7">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>43</v>
+      </c>
+      <c r="S7" t="s">
+        <v>100</v>
+      </c>
+      <c r="T7" t="s">
+        <v>101</v>
+      </c>
+      <c r="U7" t="s">
+        <v>102</v>
+      </c>
+      <c r="V7" t="s">
+        <v>57</v>
+      </c>
+      <c r="W7" t="s">
+        <v>41</v>
+      </c>
+      <c r="X7" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24">
+      <c r="A8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" t="s">
+        <v>104</v>
+      </c>
+      <c r="F8" t="s">
+        <v>106</v>
+      </c>
+      <c r="G8" t="s">
+        <v>156</v>
+      </c>
+      <c r="H8" s="1">
+        <v>44529</v>
+      </c>
+      <c r="I8" s="2">
+        <v>44529.8111689815</v>
+      </c>
+      <c r="J8" t="s">
+        <v>157</v>
+      </c>
+      <c r="K8" t="s">
+        <v>158</v>
+      </c>
+      <c r="L8" t="s">
+        <v>159</v>
+      </c>
+      <c r="M8">
+        <v>3</v>
+      </c>
+      <c r="N8">
+        <v>31.75</v>
+      </c>
+      <c r="O8">
+        <v>-95.25</v>
+      </c>
+      <c r="P8">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>43</v>
+      </c>
+      <c r="S8" t="s">
+        <v>107</v>
+      </c>
+      <c r="T8" t="s">
+        <v>108</v>
+      </c>
+      <c r="U8" t="s">
+        <v>109</v>
+      </c>
+      <c r="V8" t="s">
+        <v>36</v>
+      </c>
+      <c r="W8" t="s">
+        <v>41</v>
+      </c>
+      <c r="X8" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24">
+      <c r="A9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" t="s">
+        <v>110</v>
+      </c>
+      <c r="F9" t="s">
+        <v>112</v>
+      </c>
+      <c r="G9" t="s">
+        <v>156</v>
+      </c>
+      <c r="H9" s="1">
+        <v>44529</v>
+      </c>
+      <c r="I9" s="2">
+        <v>44529.8111689815</v>
+      </c>
+      <c r="J9" t="s">
+        <v>157</v>
+      </c>
+      <c r="K9" t="s">
+        <v>158</v>
+      </c>
+      <c r="L9" t="s">
+        <v>159</v>
+      </c>
+      <c r="M9">
+        <v>100</v>
+      </c>
+      <c r="N9">
+        <v>18.53</v>
+      </c>
+      <c r="O9">
+        <v>-1853</v>
+      </c>
+      <c r="P9">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>43</v>
+      </c>
+      <c r="S9" t="s">
+        <v>113</v>
+      </c>
+      <c r="T9" t="s">
+        <v>114</v>
+      </c>
+      <c r="U9" t="s">
+        <v>115</v>
+      </c>
+      <c r="V9" t="s">
+        <v>36</v>
+      </c>
+      <c r="W9" t="s">
+        <v>116</v>
+      </c>
+      <c r="X9" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24">
+      <c r="A10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F10" t="s">
+        <v>120</v>
+      </c>
+      <c r="G10" t="s">
+        <v>156</v>
+      </c>
+      <c r="H10" s="1">
+        <v>44529</v>
+      </c>
+      <c r="I10" s="2">
+        <v>44529.8111689815</v>
+      </c>
+      <c r="J10" t="s">
+        <v>157</v>
+      </c>
+      <c r="K10" t="s">
+        <v>158</v>
+      </c>
+      <c r="L10" t="s">
+        <v>159</v>
+      </c>
+      <c r="M10">
+        <v>60</v>
+      </c>
+      <c r="N10">
+        <v>30.33</v>
+      </c>
+      <c r="O10">
+        <v>-1819.5</v>
+      </c>
+      <c r="P10">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>43</v>
+      </c>
+      <c r="S10" t="s">
+        <v>121</v>
+      </c>
+      <c r="T10" t="s">
+        <v>122</v>
+      </c>
+      <c r="U10" t="s">
+        <v>123</v>
+      </c>
+      <c r="V10" t="s">
+        <v>36</v>
+      </c>
+      <c r="W10" t="s">
+        <v>116</v>
+      </c>
+      <c r="X10" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24">
+      <c r="A11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" t="s">
+        <v>124</v>
+      </c>
+      <c r="F11" t="s">
+        <v>126</v>
+      </c>
+      <c r="G11" t="s">
+        <v>156</v>
+      </c>
+      <c r="H11" s="1">
+        <v>44529</v>
+      </c>
+      <c r="I11" s="2">
+        <v>44529.8111689815</v>
+      </c>
+      <c r="J11" t="s">
+        <v>157</v>
+      </c>
+      <c r="K11" t="s">
+        <v>158</v>
+      </c>
+      <c r="L11" t="s">
+        <v>159</v>
+      </c>
+      <c r="M11">
+        <v>345</v>
+      </c>
+      <c r="N11">
+        <v>6.59</v>
+      </c>
+      <c r="O11">
+        <v>-2272.74</v>
+      </c>
+      <c r="P11">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>43</v>
+      </c>
+      <c r="S11" t="s">
+        <v>127</v>
+      </c>
+      <c r="T11" t="s">
+        <v>128</v>
+      </c>
+      <c r="U11" t="s">
+        <v>129</v>
+      </c>
+      <c r="V11" t="s">
+        <v>36</v>
+      </c>
+      <c r="W11" t="s">
+        <v>116</v>
+      </c>
+      <c r="X11" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="12" spans="1:24">
+      <c r="A12" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" t="s">
+        <v>130</v>
+      </c>
+      <c r="F12" t="s">
+        <v>132</v>
+      </c>
+      <c r="G12" t="s">
+        <v>156</v>
+      </c>
+      <c r="H12" s="1">
+        <v>44529</v>
+      </c>
+      <c r="I12" s="2">
+        <v>44529.8111689815</v>
+      </c>
+      <c r="J12" t="s">
+        <v>157</v>
+      </c>
+      <c r="K12" t="s">
+        <v>158</v>
+      </c>
+      <c r="L12" t="s">
+        <v>159</v>
+      </c>
+      <c r="M12">
+        <v>300</v>
+      </c>
+      <c r="N12">
+        <v>49.6</v>
+      </c>
+      <c r="O12">
+        <v>-14879.48</v>
+      </c>
+      <c r="P12">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>43</v>
+      </c>
+      <c r="S12" t="s">
+        <v>133</v>
+      </c>
+      <c r="T12" t="s">
+        <v>134</v>
+      </c>
+      <c r="U12" t="s">
+        <v>135</v>
+      </c>
+      <c r="V12" t="s">
+        <v>36</v>
+      </c>
+      <c r="W12" t="s">
+        <v>116</v>
+      </c>
+      <c r="X12" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24">
+      <c r="A13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B13" t="s">
+        <v>136</v>
+      </c>
+      <c r="F13" t="s">
+        <v>138</v>
+      </c>
+      <c r="G13" t="s">
+        <v>156</v>
+      </c>
+      <c r="H13" s="1">
+        <v>44529</v>
+      </c>
+      <c r="I13" s="2">
+        <v>44529.8111689815</v>
+      </c>
+      <c r="J13" t="s">
+        <v>157</v>
+      </c>
+      <c r="K13" t="s">
+        <v>158</v>
+      </c>
+      <c r="L13" t="s">
+        <v>159</v>
+      </c>
+      <c r="M13">
+        <v>3</v>
+      </c>
+      <c r="N13">
+        <v>179.07</v>
+      </c>
+      <c r="O13">
+        <v>-537.21</v>
+      </c>
+      <c r="P13">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>43</v>
+      </c>
+      <c r="S13" t="s">
+        <v>139</v>
+      </c>
+      <c r="T13" t="s">
+        <v>140</v>
+      </c>
+      <c r="U13" t="s">
+        <v>141</v>
+      </c>
+      <c r="V13" t="s">
+        <v>57</v>
+      </c>
+      <c r="W13" t="s">
+        <v>41</v>
+      </c>
+      <c r="X13" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="14" spans="1:24">
+      <c r="A14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" t="s">
+        <v>143</v>
+      </c>
+      <c r="F14" t="s">
+        <v>145</v>
+      </c>
+      <c r="G14" t="s">
+        <v>156</v>
+      </c>
+      <c r="H14" s="1">
+        <v>44529</v>
+      </c>
+      <c r="I14" s="2">
+        <v>44529.8111689815</v>
+      </c>
+      <c r="J14" t="s">
+        <v>157</v>
+      </c>
+      <c r="K14" t="s">
+        <v>158</v>
+      </c>
+      <c r="L14" t="s">
+        <v>159</v>
+      </c>
+      <c r="M14">
+        <v>300</v>
+      </c>
+      <c r="N14">
+        <v>14.25</v>
+      </c>
+      <c r="O14">
+        <v>-4273.5</v>
+      </c>
+      <c r="P14">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>43</v>
+      </c>
+      <c r="S14" t="s">
+        <v>38</v>
+      </c>
+      <c r="T14" t="s">
+        <v>39</v>
+      </c>
+      <c r="U14" t="s">
+        <v>40</v>
+      </c>
+      <c r="V14" t="s">
+        <v>37</v>
+      </c>
+      <c r="W14" t="s">
+        <v>41</v>
+      </c>
+      <c r="X14" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:U9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:21">
+      <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" t="s">
+        <v>160</v>
+      </c>
+      <c r="H1" t="s">
+        <v>161</v>
+      </c>
+      <c r="I1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J1" t="s">
+        <v>16</v>
+      </c>
+      <c r="K1" t="s">
+        <v>15</v>
+      </c>
+      <c r="L1" t="s">
+        <v>162</v>
+      </c>
+      <c r="M1" t="s">
+        <v>163</v>
+      </c>
+      <c r="N1" t="s">
+        <v>164</v>
+      </c>
+      <c r="O1" t="s">
+        <v>165</v>
+      </c>
+      <c r="P1" t="s">
+        <v>166</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>167</v>
+      </c>
+      <c r="R1" t="s">
+        <v>23</v>
+      </c>
+      <c r="S1" t="s">
+        <v>24</v>
+      </c>
+      <c r="T1" t="s">
+        <v>25</v>
+      </c>
+      <c r="U1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2" t="s">
+        <v>168</v>
+      </c>
+      <c r="E2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G2" t="s">
+        <v>169</v>
+      </c>
+      <c r="H2" t="s">
+        <v>170</v>
+      </c>
+      <c r="I2">
+        <v>-4.44</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0.71594</v>
+      </c>
+      <c r="L2" s="1">
+        <v>44561</v>
+      </c>
+      <c r="M2" t="s">
+        <v>171</v>
+      </c>
+      <c r="N2" t="s">
+        <v>172</v>
+      </c>
+      <c r="O2">
+        <v>300</v>
+      </c>
+      <c r="P2" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q2">
+        <v>25</v>
+      </c>
+      <c r="R2" t="s">
+        <v>38</v>
+      </c>
+      <c r="S2" t="s">
+        <v>39</v>
+      </c>
+      <c r="T2" t="s">
+        <v>40</v>
+      </c>
+      <c r="U2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21">
+      <c r="A3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" t="s">
+        <v>173</v>
+      </c>
+      <c r="E3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G3" t="s">
+        <v>174</v>
+      </c>
+      <c r="H3" t="s">
+        <v>175</v>
+      </c>
+      <c r="I3">
+        <v>17.74</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0.71594</v>
+      </c>
+      <c r="L3" s="1">
+        <v>44561</v>
+      </c>
+      <c r="M3" t="s">
+        <v>171</v>
+      </c>
+      <c r="N3" t="s">
+        <v>172</v>
+      </c>
+      <c r="O3">
+        <v>300</v>
+      </c>
+      <c r="P3" t="s">
+        <v>176</v>
+      </c>
+      <c r="R3" t="s">
+        <v>38</v>
+      </c>
+      <c r="S3" t="s">
+        <v>39</v>
+      </c>
+      <c r="T3" t="s">
+        <v>40</v>
+      </c>
+      <c r="U3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21">
+      <c r="A4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G4" t="s">
+        <v>47</v>
+      </c>
+      <c r="H4" t="s">
+        <v>177</v>
+      </c>
+      <c r="I4">
+        <v>-0.7</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4" s="1">
+        <v>44544</v>
+      </c>
+      <c r="M4" t="s">
+        <v>172</v>
+      </c>
+      <c r="N4" t="s">
+        <v>172</v>
+      </c>
+      <c r="P4" t="s">
+        <v>172</v>
+      </c>
+      <c r="U4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21">
+      <c r="A5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" t="s">
+        <v>178</v>
+      </c>
+      <c r="E5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G5" t="s">
+        <v>169</v>
+      </c>
+      <c r="H5" t="s">
+        <v>170</v>
+      </c>
+      <c r="I5">
+        <v>-4.11</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0.633124</v>
+      </c>
+      <c r="L5" s="1">
+        <v>44530</v>
+      </c>
+      <c r="M5" t="s">
+        <v>179</v>
+      </c>
+      <c r="N5" t="s">
+        <v>172</v>
+      </c>
+      <c r="P5" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q5">
+        <v>25</v>
+      </c>
+      <c r="R5" t="s">
+        <v>38</v>
+      </c>
+      <c r="S5" t="s">
+        <v>39</v>
+      </c>
+      <c r="T5" t="s">
+        <v>40</v>
+      </c>
+      <c r="U5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21">
+      <c r="A6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" t="s">
+        <v>180</v>
+      </c>
+      <c r="E6" t="s">
+        <v>49</v>
+      </c>
+      <c r="F6" t="s">
+        <v>35</v>
+      </c>
+      <c r="G6" t="s">
+        <v>174</v>
+      </c>
+      <c r="H6" t="s">
+        <v>175</v>
+      </c>
+      <c r="I6">
+        <v>16.43</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0.633124</v>
+      </c>
+      <c r="L6" s="1">
+        <v>44530</v>
+      </c>
+      <c r="M6" t="s">
+        <v>179</v>
+      </c>
+      <c r="N6" t="s">
+        <v>172</v>
+      </c>
+      <c r="P6" t="s">
+        <v>176</v>
+      </c>
+      <c r="R6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S6" t="s">
+        <v>39</v>
+      </c>
+      <c r="T6" t="s">
+        <v>40</v>
+      </c>
+      <c r="U6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21">
+      <c r="A7" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" t="s">
+        <v>51</v>
+      </c>
+      <c r="F7" t="s">
+        <v>52</v>
+      </c>
+      <c r="G7" t="s">
+        <v>46</v>
+      </c>
+      <c r="H7" t="s">
+        <v>181</v>
+      </c>
+      <c r="I7">
+        <v>848.79</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0.639606</v>
+      </c>
+      <c r="L7" s="1">
+        <v>44529</v>
+      </c>
+      <c r="M7" t="s">
+        <v>172</v>
+      </c>
+      <c r="N7" t="s">
+        <v>172</v>
+      </c>
+      <c r="P7" t="s">
+        <v>172</v>
+      </c>
+      <c r="U7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21">
+      <c r="A8" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" t="s">
+        <v>56</v>
+      </c>
+      <c r="F8" t="s">
+        <v>52</v>
+      </c>
+      <c r="G8" t="s">
+        <v>46</v>
+      </c>
+      <c r="H8" t="s">
+        <v>181</v>
+      </c>
+      <c r="I8">
+        <v>844.92</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0.91399</v>
+      </c>
+      <c r="L8" s="1">
+        <v>44529</v>
+      </c>
+      <c r="M8" t="s">
+        <v>172</v>
+      </c>
+      <c r="N8" t="s">
+        <v>172</v>
+      </c>
+      <c r="P8" t="s">
+        <v>172</v>
+      </c>
+      <c r="U8" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21">
+      <c r="A9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" t="s">
+        <v>59</v>
+      </c>
+      <c r="F9" t="s">
+        <v>52</v>
+      </c>
+      <c r="G9" t="s">
+        <v>46</v>
+      </c>
+      <c r="H9" t="s">
+        <v>181</v>
+      </c>
+      <c r="I9">
+        <v>7960.26</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>1</v>
+      </c>
+      <c r="L9" s="1">
+        <v>44529</v>
+      </c>
+      <c r="M9" t="s">
+        <v>172</v>
+      </c>
+      <c r="N9" t="s">
+        <v>172</v>
+      </c>
+      <c r="P9" t="s">
+        <v>172</v>
+      </c>
+      <c r="U9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>